<commit_message>
Premium UI Upgrade: Navy/Cyan theme with smooth animations and enhanced ticket persistence
</commit_message>
<xml_diff>
--- a/data/bookings.xlsx
+++ b/data/bookings.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -464,39 +464,219 @@
           <t>Booking_Date</t>
         </is>
       </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>45 Ahamad</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>7259869733</v>
+      </c>
+      <c r="C2" t="n">
+        <v>5</v>
+      </c>
+      <c r="D2" t="n">
+        <v>50</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>1756722415</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>2025-09-16 19:55:57</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>45 Ahamad</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>8762069113</v>
+      </c>
+      <c r="C3" t="n">
+        <v>6</v>
+      </c>
+      <c r="D3" t="n">
+        <v>50</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>524463279344</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>2025-09-16 19:59:22</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
           <t>chamma</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>9353539771</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>0005, 0006</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>10</v>
-      </c>
-      <c r="E2" t="inlineStr">
+      <c r="B4" t="n">
+        <v>7259869733</v>
+      </c>
+      <c r="C4" t="n">
+        <v>236</v>
+      </c>
+      <c r="D4" t="n">
+        <v>50</v>
+      </c>
+      <c r="E4" t="inlineStr">
         <is>
           <t>Paid</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>524472913877</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>2025-09-02 00:27:03</t>
+      <c r="F4" t="n">
+        <v>1756727320</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>2025-09-16 20:01:49</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Ahamad Sharvan</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>9353539771</v>
+      </c>
+      <c r="C5" t="n">
+        <v>14</v>
+      </c>
+      <c r="D5" t="n">
+        <v>50</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>123456789123</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>2025-09-16 20:10:40</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ahamad </t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>6356487201</v>
+      </c>
+      <c r="C6" t="n">
+        <v>13</v>
+      </c>
+      <c r="D6" t="n">
+        <v>50</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>123456789123</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>2025-09-16 20:14:06</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ahamad Sharvan </t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>9845841795</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>0018</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>50</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>542548525489</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>2025-09-17 22:55:47</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Pending</t>
         </is>
       </c>
     </row>

</xml_diff>